<commit_message>
Regenerate CHD reference outputs: AlphaMissense fix + relaxed/pathonly thresholds
Regenerated with scripts/apply_chd_concordance.py and scripts/collapse_chd.py.

chd_concordance_results_FIXED.csv
  Correct 15 transposed AlphaMissense rows (kpna1 x2, kpna6 x4, tcf7l1 x9).
  This flips am_vote for the two likely-pathogenic calls, raising KPNA6 K424N
  to 3/4 and I498T to 4/4 strict concordance (both were suppressed by the
  transposition). Append 10 pathogenic-only columns. No structural, ddG, tier,
  or mechanism value changes.

chd_concordance_collapsed.csv, MAVIS_CHD_concordance_collapsed.xlsx
  Correct AlphaMissense class/score for the 15 variants; update am_hit and
  concordance for KPNA6 K424N and I498T; append relaxed and pathogenic-only
  concordance columns. All curated columns and the ZIC3_controls_detail /
  Notes sheets preserved.
</commit_message>
<xml_diff>
--- a/reference_outputs/MAVIS_CHD_concordance_collapsed.xlsx
+++ b/reference_outputs/MAVIS_CHD_concordance_collapsed.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W145"/>
+  <dimension ref="A1:AC145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -501,6 +501,12 @@
     <col width="15" customWidth="1" min="21" max="21"/>
     <col width="13" customWidth="1" min="22" max="22"/>
     <col width="62" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -619,6 +625,36 @@
           <t>control_citation</t>
         </is>
       </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>conc_relaxed_n</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>conc_relaxed_denom</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>concordance_relaxed</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>conc_pathonly_n</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>conc_pathonly_denom</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>concordance_pathonly</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -708,6 +744,28 @@
           <t>Ware 2004 (DOI 10.1086/380998); ClinVar RCV000012190; rs104894961</t>
         </is>
       </c>
+      <c r="X2" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="AA2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -797,6 +855,28 @@
           <t>Sci Rep 2018 (PMID 30120289); c.890G&gt;T — not in ClinVar</t>
         </is>
       </c>
+      <c r="X3" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="AA3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -886,6 +966,28 @@
           <t>Cowan 2014 (PMID 24123890)</t>
         </is>
       </c>
+      <c r="X4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="AA4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -975,6 +1077,28 @@
           <t>Cowan 2014 (PMID 24123890); OMIM/ClinVar RCV000012186 (as Thr325Met)</t>
         </is>
       </c>
+      <c r="X5" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="AA5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1064,6 +1188,28 @@
           <t>Ware 2004 (DOI 10.1086/380998); ClinVar RCV000012191; rs104894962</t>
         </is>
       </c>
+      <c r="X6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="AA6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1153,6 +1299,28 @@
           <t>D'Alessandro 2013 (PMID 23427188); c.841C&gt;T — not in ClinVar</t>
         </is>
       </c>
+      <c r="X7" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="AA7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1242,6 +1410,28 @@
           <t>Cowan 2014 (PMID 24123890)</t>
         </is>
       </c>
+      <c r="X8" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="AA8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1331,6 +1521,28 @@
           <t>Cowan 2014 (PMID 24123890)</t>
         </is>
       </c>
+      <c r="X9" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="AA9" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1420,6 +1632,28 @@
           <t>Cowan 2014 (PMID 24123890); NLS/NES mech. Bedard 2006 (DOI 10.1093/hmg/ddl461)</t>
         </is>
       </c>
+      <c r="X10" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="AA10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1513,6 +1747,28 @@
           <t>Cowan 2014 (PMID 24123890) — atypical, increased transactivation</t>
         </is>
       </c>
+      <c r="X11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1606,6 +1862,28 @@
           <t>Cowan 2014 (PMID 24123890) — susceptibility allele, incomplete penetrance</t>
         </is>
       </c>
+      <c r="X12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1691,6 +1969,28 @@
         <v>3</v>
       </c>
       <c r="W13" s="2" t="inlineStr"/>
+      <c r="X13" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="AA13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1776,6 +2076,28 @@
         <v>5</v>
       </c>
       <c r="W14" s="2" t="inlineStr"/>
+      <c r="X14" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="AA14" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1861,6 +2183,28 @@
         <v>5.5</v>
       </c>
       <c r="W15" s="2" t="inlineStr"/>
+      <c r="X15" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="AA15" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1902,18 +2246,18 @@
         <v>1</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="N16" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O16" s="2" t="n">
         <v>4</v>
@@ -1929,10 +2273,12 @@
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="S16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="n">
+        <v>0.8778</v>
+      </c>
       <c r="T16" s="2" t="inlineStr">
         <is>
-          <t>0.8778</t>
+          <t>likely_pathogenic</t>
         </is>
       </c>
       <c r="U16" s="2" t="inlineStr">
@@ -1944,6 +2290,28 @@
         <v>4</v>
       </c>
       <c r="W16" s="2" t="inlineStr"/>
+      <c r="X16" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="AA16" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2029,6 +2397,28 @@
         <v>5.5</v>
       </c>
       <c r="W17" s="2" t="inlineStr"/>
+      <c r="X17" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="AA17" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2114,6 +2504,28 @@
         <v>6.5</v>
       </c>
       <c r="W18" s="2" t="inlineStr"/>
+      <c r="X18" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="AA18" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2199,6 +2611,28 @@
         <v>3.5</v>
       </c>
       <c r="W19" s="2" t="inlineStr"/>
+      <c r="X19" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="AA19" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2240,18 +2674,18 @@
         <v>0</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="N20" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O20" s="2" t="n">
         <v>4</v>
@@ -2267,10 +2701,12 @@
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="S20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="n">
+        <v>0.6877</v>
+      </c>
       <c r="T20" s="2" t="inlineStr">
         <is>
-          <t>0.6877</t>
+          <t>likely_pathogenic</t>
         </is>
       </c>
       <c r="U20" s="2" t="inlineStr">
@@ -2282,6 +2718,28 @@
         <v>3</v>
       </c>
       <c r="W20" s="2" t="inlineStr"/>
+      <c r="X20" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="AA20" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2367,6 +2825,28 @@
         <v>1.4</v>
       </c>
       <c r="W21" s="2" t="inlineStr"/>
+      <c r="X21" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="AA21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2452,6 +2932,28 @@
         <v>6</v>
       </c>
       <c r="W22" s="2" t="inlineStr"/>
+      <c r="X22" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="AA22" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2537,6 +3039,28 @@
         <v>4</v>
       </c>
       <c r="W23" s="2" t="inlineStr"/>
+      <c r="X23" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
+      <c r="AA23" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2622,6 +3146,28 @@
         <v>3</v>
       </c>
       <c r="W24" s="2" t="inlineStr"/>
+      <c r="X24" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
+      <c r="AA24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2707,6 +3253,28 @@
         <v>4</v>
       </c>
       <c r="W25" s="2" t="inlineStr"/>
+      <c r="X25" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
+      <c r="AA25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2792,6 +3360,28 @@
         <v>2</v>
       </c>
       <c r="W26" s="2" t="inlineStr"/>
+      <c r="X26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
+      <c r="AA26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2877,6 +3467,28 @@
         <v>0</v>
       </c>
       <c r="W27" s="2" t="inlineStr"/>
+      <c r="X27" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="AA27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2962,6 +3574,28 @@
         <v>2</v>
       </c>
       <c r="W28" s="2" t="inlineStr"/>
+      <c r="X28" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
+      <c r="AA28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB28" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3047,6 +3681,28 @@
         <v>0</v>
       </c>
       <c r="W29" s="2" t="inlineStr"/>
+      <c r="X29" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3132,6 +3788,28 @@
         <v>0</v>
       </c>
       <c r="W30" s="2" t="inlineStr"/>
+      <c r="X30" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3217,6 +3895,28 @@
         <v>0.4</v>
       </c>
       <c r="W31" s="2" t="inlineStr"/>
+      <c r="X31" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3302,6 +4002,28 @@
         <v>0</v>
       </c>
       <c r="W32" s="2" t="inlineStr"/>
+      <c r="X32" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3370,10 +4092,12 @@
           <t>Tier 3</t>
         </is>
       </c>
-      <c r="S33" s="2" t="inlineStr"/>
+      <c r="S33" s="2" t="n">
+        <v>0.4622</v>
+      </c>
       <c r="T33" s="2" t="inlineStr">
         <is>
-          <t>0.4622</t>
+          <t>ambiguous</t>
         </is>
       </c>
       <c r="U33" s="2" t="inlineStr">
@@ -3385,6 +4109,28 @@
         <v>2</v>
       </c>
       <c r="W33" s="2" t="inlineStr"/>
+      <c r="X33" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
+      <c r="AA33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB33" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3453,10 +4199,12 @@
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="S34" s="2" t="inlineStr"/>
+      <c r="S34" s="2" t="n">
+        <v>0.3399</v>
+      </c>
       <c r="T34" s="2" t="inlineStr">
         <is>
-          <t>0.3399</t>
+          <t>likely_benign</t>
         </is>
       </c>
       <c r="U34" s="2" t="inlineStr">
@@ -3468,6 +4216,28 @@
         <v>3</v>
       </c>
       <c r="W34" s="2" t="inlineStr"/>
+      <c r="X34" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="AA34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB34" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3553,6 +4323,28 @@
         <v>0</v>
       </c>
       <c r="W35" s="2" t="inlineStr"/>
+      <c r="X35" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB35" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3638,6 +4430,28 @@
         <v>3</v>
       </c>
       <c r="W36" s="2" t="inlineStr"/>
+      <c r="X36" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
+      <c r="AA36" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB36" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3723,6 +4537,28 @@
         <v>2</v>
       </c>
       <c r="W37" s="2" t="inlineStr"/>
+      <c r="X37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
+      <c r="AA37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB37" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3808,6 +4644,28 @@
         <v>0</v>
       </c>
       <c r="W38" s="2" t="inlineStr"/>
+      <c r="X38" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="AA38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB38" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3893,6 +4751,28 @@
         <v>1</v>
       </c>
       <c r="W39" s="2" t="inlineStr"/>
+      <c r="X39" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
+      <c r="AA39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3978,6 +4858,28 @@
         <v>0.7</v>
       </c>
       <c r="W40" s="2" t="inlineStr"/>
+      <c r="X40" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
+      <c r="AA40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB40" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4063,6 +4965,28 @@
         <v>0</v>
       </c>
       <c r="W41" s="2" t="inlineStr"/>
+      <c r="X41" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="AA41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB41" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC41" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4148,6 +5072,28 @@
         <v>0.4</v>
       </c>
       <c r="W42" s="2" t="inlineStr"/>
+      <c r="X42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y42" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB42" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4233,6 +5179,28 @@
         <v>0</v>
       </c>
       <c r="W43" s="2" t="inlineStr"/>
+      <c r="X43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB43" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC43" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4318,6 +5286,28 @@
         <v>1</v>
       </c>
       <c r="W44" s="2" t="inlineStr"/>
+      <c r="X44" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
+      <c r="AA44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB44" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC44" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4403,6 +5393,28 @@
         <v>2</v>
       </c>
       <c r="W45" s="2" t="inlineStr"/>
+      <c r="X45" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
+      <c r="AA45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB45" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC45" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4488,6 +5500,28 @@
         <v>1</v>
       </c>
       <c r="W46" s="2" t="inlineStr"/>
+      <c r="X46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
+      <c r="AA46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB46" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC46" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4573,6 +5607,28 @@
         <v>1</v>
       </c>
       <c r="W47" s="2" t="inlineStr"/>
+      <c r="X47" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
+      <c r="AA47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB47" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC47" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4658,6 +5714,28 @@
         <v>0</v>
       </c>
       <c r="W48" s="2" t="inlineStr"/>
+      <c r="X48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y48" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB48" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC48" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4743,6 +5821,28 @@
         <v>1</v>
       </c>
       <c r="W49" s="2" t="inlineStr"/>
+      <c r="X49" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y49" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
+      <c r="AA49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB49" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC49" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4828,6 +5928,28 @@
         <v>1</v>
       </c>
       <c r="W50" s="2" t="inlineStr"/>
+      <c r="X50" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y50" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
+      <c r="AA50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB50" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC50" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4913,6 +6035,28 @@
         <v>0</v>
       </c>
       <c r="W51" s="2" t="inlineStr"/>
+      <c r="X51" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y51" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB51" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC51" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4998,6 +6142,28 @@
         <v>0</v>
       </c>
       <c r="W52" s="2" t="inlineStr"/>
+      <c r="X52" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y52" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z52" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="AA52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB52" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC52" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -5083,6 +6249,28 @@
         <v>0</v>
       </c>
       <c r="W53" s="2" t="inlineStr"/>
+      <c r="X53" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y53" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="AA53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB53" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC53" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -5168,6 +6356,28 @@
         <v>0</v>
       </c>
       <c r="W54" s="2" t="inlineStr"/>
+      <c r="X54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y54" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB54" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC54" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -5253,6 +6463,28 @@
         <v>0</v>
       </c>
       <c r="W55" s="2" t="inlineStr"/>
+      <c r="X55" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y55" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z55" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
+      <c r="AA55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB55" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC55" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -5338,6 +6570,28 @@
         <v>0</v>
       </c>
       <c r="W56" s="2" t="inlineStr"/>
+      <c r="X56" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y56" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z56" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB56" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC56" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -5423,6 +6677,28 @@
         <v>0.4</v>
       </c>
       <c r="W57" s="2" t="inlineStr"/>
+      <c r="X57" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y57" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z57" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB57" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC57" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -5508,6 +6784,28 @@
         <v>0.4</v>
       </c>
       <c r="W58" s="2" t="inlineStr"/>
+      <c r="X58" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y58" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z58" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB58" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC58" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -5593,6 +6891,28 @@
         <v>0</v>
       </c>
       <c r="W59" s="2" t="inlineStr"/>
+      <c r="X59" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y59" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z59" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
+      <c r="AA59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB59" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC59" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5678,6 +6998,28 @@
         <v>0</v>
       </c>
       <c r="W60" s="2" t="inlineStr"/>
+      <c r="X60" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y60" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z60" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB60" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC60" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5763,6 +7105,28 @@
         <v>0</v>
       </c>
       <c r="W61" s="2" t="inlineStr"/>
+      <c r="X61" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y61" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z61" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB61" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC61" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5848,6 +7212,28 @@
         <v>0</v>
       </c>
       <c r="W62" s="2" t="inlineStr"/>
+      <c r="X62" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y62" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z62" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB62" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC62" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5933,6 +7319,28 @@
         <v>0</v>
       </c>
       <c r="W63" s="2" t="inlineStr"/>
+      <c r="X63" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y63" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z63" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB63" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC63" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -6018,6 +7426,28 @@
         <v>0</v>
       </c>
       <c r="W64" s="2" t="inlineStr"/>
+      <c r="X64" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y64" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z64" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB64" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC64" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -6103,6 +7533,28 @@
         <v>0</v>
       </c>
       <c r="W65" s="2" t="inlineStr"/>
+      <c r="X65" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y65" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z65" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB65" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC65" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -6188,6 +7640,28 @@
         <v>0</v>
       </c>
       <c r="W66" s="2" t="inlineStr"/>
+      <c r="X66" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y66" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z66" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB66" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC66" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -6273,6 +7747,28 @@
         <v>0</v>
       </c>
       <c r="W67" s="2" t="inlineStr"/>
+      <c r="X67" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y67" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB67" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC67" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -6358,6 +7854,28 @@
         <v>0</v>
       </c>
       <c r="W68" s="2" t="inlineStr"/>
+      <c r="X68" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y68" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z68" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB68" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC68" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -6443,6 +7961,28 @@
         <v>0</v>
       </c>
       <c r="W69" s="2" t="inlineStr"/>
+      <c r="X69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y69" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z69" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB69" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC69" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -6528,6 +8068,28 @@
         <v>0</v>
       </c>
       <c r="W70" s="2" t="inlineStr"/>
+      <c r="X70" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y70" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z70" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB70" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC70" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -6613,6 +8175,28 @@
         <v>0</v>
       </c>
       <c r="W71" s="2" t="inlineStr"/>
+      <c r="X71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB71" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC71" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -6698,6 +8282,28 @@
         <v>0</v>
       </c>
       <c r="W72" s="2" t="inlineStr"/>
+      <c r="X72" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y72" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z72" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB72" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC72" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -6783,6 +8389,28 @@
         <v>0</v>
       </c>
       <c r="W73" s="2" t="inlineStr"/>
+      <c r="X73" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y73" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z73" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB73" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC73" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -6868,6 +8496,28 @@
         <v>0</v>
       </c>
       <c r="W74" s="2" t="inlineStr"/>
+      <c r="X74" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y74" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z74" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB74" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC74" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -6953,6 +8603,28 @@
         <v>0</v>
       </c>
       <c r="W75" s="2" t="inlineStr"/>
+      <c r="X75" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y75" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z75" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB75" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC75" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -7038,6 +8710,28 @@
         <v>0</v>
       </c>
       <c r="W76" s="2" t="inlineStr"/>
+      <c r="X76" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y76" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z76" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB76" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC76" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -7123,6 +8817,28 @@
         <v>0</v>
       </c>
       <c r="W77" s="2" t="inlineStr"/>
+      <c r="X77" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y77" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z77" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB77" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC77" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -7208,6 +8924,28 @@
         <v>0</v>
       </c>
       <c r="W78" s="2" t="inlineStr"/>
+      <c r="X78" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y78" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z78" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB78" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC78" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -7293,6 +9031,28 @@
         <v>0</v>
       </c>
       <c r="W79" s="2" t="inlineStr"/>
+      <c r="X79" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z79" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC79" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -7378,6 +9138,28 @@
         <v>0</v>
       </c>
       <c r="W80" s="2" t="inlineStr"/>
+      <c r="X80" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y80" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z80" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC80" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -7463,6 +9245,28 @@
         <v>0</v>
       </c>
       <c r="W81" s="2" t="inlineStr"/>
+      <c r="X81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y81" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z81" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB81" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC81" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -7548,6 +9352,28 @@
         <v>1.2</v>
       </c>
       <c r="W82" s="2" t="inlineStr"/>
+      <c r="X82" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y82" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z82" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB82" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC82" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -7633,6 +9459,28 @@
         <v>0</v>
       </c>
       <c r="W83" s="2" t="inlineStr"/>
+      <c r="X83" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y83" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z83" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB83" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC83" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -7718,6 +9566,28 @@
         <v>0.8</v>
       </c>
       <c r="W84" s="2" t="inlineStr"/>
+      <c r="X84" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y84" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z84" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB84" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC84" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -7803,6 +9673,28 @@
         <v>0</v>
       </c>
       <c r="W85" s="2" t="inlineStr"/>
+      <c r="X85" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y85" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z85" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB85" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC85" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -7888,6 +9780,28 @@
         <v>0</v>
       </c>
       <c r="W86" s="2" t="inlineStr"/>
+      <c r="X86" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y86" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z86" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB86" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC86" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -7956,10 +9870,12 @@
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="S87" s="2" t="inlineStr"/>
+      <c r="S87" s="2" t="n">
+        <v>0.0728</v>
+      </c>
       <c r="T87" s="2" t="inlineStr">
         <is>
-          <t>0.0728</t>
+          <t>likely_benign</t>
         </is>
       </c>
       <c r="U87" s="2" t="inlineStr">
@@ -7971,6 +9887,28 @@
         <v>0</v>
       </c>
       <c r="W87" s="2" t="inlineStr"/>
+      <c r="X87" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y87" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z87" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB87" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC87" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -8039,10 +9977,12 @@
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="S88" s="2" t="inlineStr"/>
+      <c r="S88" s="2" t="n">
+        <v>0.1991</v>
+      </c>
       <c r="T88" s="2" t="inlineStr">
         <is>
-          <t>0.1991</t>
+          <t>likely_benign</t>
         </is>
       </c>
       <c r="U88" s="2" t="inlineStr">
@@ -8054,6 +9994,28 @@
         <v>0</v>
       </c>
       <c r="W88" s="2" t="inlineStr"/>
+      <c r="X88" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y88" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z88" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA88" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB88" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC88" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -8139,6 +10101,28 @@
         <v>0</v>
       </c>
       <c r="W89" s="2" t="inlineStr"/>
+      <c r="X89" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y89" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z89" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
+      <c r="AA89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB89" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC89" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -8224,6 +10208,28 @@
         <v>1.4</v>
       </c>
       <c r="W90" s="2" t="inlineStr"/>
+      <c r="X90" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y90" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z90" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
+      <c r="AA90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB90" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC90" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -8309,6 +10315,28 @@
         <v>2</v>
       </c>
       <c r="W91" s="2" t="inlineStr"/>
+      <c r="X91" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y91" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z91" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
+      <c r="AA91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB91" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC91" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -8394,6 +10422,28 @@
         <v>1</v>
       </c>
       <c r="W92" s="2" t="inlineStr"/>
+      <c r="X92" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y92" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z92" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
+      <c r="AA92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB92" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC92" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -8479,6 +10529,28 @@
         <v>0</v>
       </c>
       <c r="W93" s="2" t="inlineStr"/>
+      <c r="X93" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y93" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z93" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA93" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB93" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC93" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -8564,6 +10636,28 @@
         <v>0</v>
       </c>
       <c r="W94" s="2" t="inlineStr"/>
+      <c r="X94" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y94" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z94" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB94" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC94" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -8649,6 +10743,28 @@
         <v>0</v>
       </c>
       <c r="W95" s="2" t="inlineStr"/>
+      <c r="X95" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y95" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z95" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB95" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC95" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -8734,6 +10850,28 @@
         <v>0</v>
       </c>
       <c r="W96" s="2" t="inlineStr"/>
+      <c r="X96" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y96" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="AA96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB96" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC96" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -8819,6 +10957,28 @@
         <v>0</v>
       </c>
       <c r="W97" s="2" t="inlineStr"/>
+      <c r="X97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y97" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z97" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA97" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB97" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC97" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -8904,6 +11064,28 @@
         <v>0</v>
       </c>
       <c r="W98" s="2" t="inlineStr"/>
+      <c r="X98" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y98" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z98" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB98" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC98" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -8989,6 +11171,28 @@
         <v>0</v>
       </c>
       <c r="W99" s="2" t="inlineStr"/>
+      <c r="X99" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y99" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB99" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC99" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -9074,6 +11278,28 @@
         <v>0</v>
       </c>
       <c r="W100" s="2" t="inlineStr"/>
+      <c r="X100" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y100" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z100" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA100" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB100" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC100" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -9159,6 +11385,28 @@
         <v>0</v>
       </c>
       <c r="W101" s="2" t="inlineStr"/>
+      <c r="X101" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y101" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z101" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB101" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC101" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -9244,6 +11492,28 @@
         <v>0</v>
       </c>
       <c r="W102" s="2" t="inlineStr"/>
+      <c r="X102" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y102" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z102" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB102" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC102" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -9329,6 +11599,28 @@
         <v>0</v>
       </c>
       <c r="W103" s="2" t="inlineStr"/>
+      <c r="X103" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y103" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z103" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB103" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC103" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -9414,6 +11706,28 @@
         <v>0</v>
       </c>
       <c r="W104" s="2" t="inlineStr"/>
+      <c r="X104" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y104" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z104" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB104" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC104" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -9499,6 +11813,28 @@
         <v>0</v>
       </c>
       <c r="W105" s="2" t="inlineStr"/>
+      <c r="X105" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y105" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z105" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB105" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC105" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -9584,6 +11920,28 @@
         <v>0</v>
       </c>
       <c r="W106" s="2" t="inlineStr"/>
+      <c r="X106" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y106" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z106" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB106" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC106" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -9669,6 +12027,28 @@
         <v>0</v>
       </c>
       <c r="W107" s="2" t="inlineStr"/>
+      <c r="X107" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y107" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z107" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB107" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC107" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -9754,6 +12134,28 @@
         <v>0</v>
       </c>
       <c r="W108" s="2" t="inlineStr"/>
+      <c r="X108" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y108" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z108" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB108" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC108" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -9839,6 +12241,28 @@
         <v>0</v>
       </c>
       <c r="W109" s="2" t="inlineStr"/>
+      <c r="X109" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y109" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z109" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB109" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC109" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -9924,6 +12348,28 @@
         <v>0</v>
       </c>
       <c r="W110" s="2" t="inlineStr"/>
+      <c r="X110" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y110" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z110" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB110" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC110" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -10009,6 +12455,28 @@
         <v>0.8</v>
       </c>
       <c r="W111" s="2" t="inlineStr"/>
+      <c r="X111" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y111" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z111" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA111" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB111" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC111" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -10094,6 +12562,28 @@
         <v>0</v>
       </c>
       <c r="W112" s="2" t="inlineStr"/>
+      <c r="X112" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y112" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z112" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA112" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB112" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC112" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -10179,6 +12669,28 @@
         <v>0</v>
       </c>
       <c r="W113" s="2" t="inlineStr"/>
+      <c r="X113" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y113" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z113" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="AA113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB113" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC113" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -10264,6 +12776,28 @@
         <v>0.7</v>
       </c>
       <c r="W114" s="2" t="inlineStr"/>
+      <c r="X114" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y114" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z114" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
+      <c r="AA114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB114" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC114" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -10349,6 +12883,28 @@
         <v>0.4</v>
       </c>
       <c r="W115" s="2" t="inlineStr"/>
+      <c r="X115" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y115" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z115" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA115" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB115" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC115" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -10434,6 +12990,28 @@
         <v>0</v>
       </c>
       <c r="W116" s="2" t="inlineStr"/>
+      <c r="X116" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y116" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z116" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA116" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB116" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC116" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -10519,6 +13097,28 @@
         <v>0</v>
       </c>
       <c r="W117" s="2" t="inlineStr"/>
+      <c r="X117" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y117" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z117" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA117" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB117" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC117" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -10604,6 +13204,28 @@
         <v>0</v>
       </c>
       <c r="W118" s="2" t="inlineStr"/>
+      <c r="X118" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y118" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z118" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA118" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB118" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC118" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -10689,6 +13311,28 @@
         <v>0</v>
       </c>
       <c r="W119" s="2" t="inlineStr"/>
+      <c r="X119" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y119" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z119" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA119" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB119" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC119" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -10774,6 +13418,28 @@
         <v>0</v>
       </c>
       <c r="W120" s="2" t="inlineStr"/>
+      <c r="X120" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y120" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z120" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA120" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB120" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC120" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -10859,6 +13525,28 @@
         <v>0</v>
       </c>
       <c r="W121" s="2" t="inlineStr"/>
+      <c r="X121" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y121" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z121" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA121" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB121" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC121" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -10944,6 +13632,28 @@
         <v>0</v>
       </c>
       <c r="W122" s="2" t="inlineStr"/>
+      <c r="X122" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y122" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z122" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA122" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB122" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC122" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -11029,6 +13739,28 @@
         <v>0</v>
       </c>
       <c r="W123" s="2" t="inlineStr"/>
+      <c r="X123" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y123" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z123" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA123" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB123" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC123" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -11114,6 +13846,28 @@
         <v>0</v>
       </c>
       <c r="W124" s="2" t="inlineStr"/>
+      <c r="X124" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y124" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z124" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA124" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB124" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC124" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -11199,6 +13953,28 @@
         <v>0</v>
       </c>
       <c r="W125" s="2" t="inlineStr"/>
+      <c r="X125" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y125" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z125" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA125" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB125" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC125" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -11284,6 +14060,28 @@
         <v>0</v>
       </c>
       <c r="W126" s="2" t="inlineStr"/>
+      <c r="X126" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y126" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z126" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB126" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC126" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -11369,6 +14167,28 @@
         <v>0</v>
       </c>
       <c r="W127" s="2" t="inlineStr"/>
+      <c r="X127" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y127" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z127" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
+      <c r="AA127" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB127" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC127" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -11437,10 +14257,12 @@
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="S128" s="2" t="inlineStr"/>
+      <c r="S128" s="2" t="n">
+        <v>0.1203</v>
+      </c>
       <c r="T128" s="2" t="inlineStr">
         <is>
-          <t>0.1203</t>
+          <t>likely_benign</t>
         </is>
       </c>
       <c r="U128" s="2" t="inlineStr">
@@ -11452,6 +14274,28 @@
         <v>0</v>
       </c>
       <c r="W128" s="2" t="inlineStr"/>
+      <c r="X128" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y128" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z128" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA128" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB128" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC128" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -11520,10 +14364,12 @@
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="S129" s="2" t="inlineStr"/>
+      <c r="S129" s="2" t="n">
+        <v>0.0974</v>
+      </c>
       <c r="T129" s="2" t="inlineStr">
         <is>
-          <t>0.0974</t>
+          <t>likely_benign</t>
         </is>
       </c>
       <c r="U129" s="2" t="inlineStr">
@@ -11535,6 +14381,28 @@
         <v>0</v>
       </c>
       <c r="W129" s="2" t="inlineStr"/>
+      <c r="X129" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y129" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z129" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA129" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB129" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC129" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -11603,10 +14471,12 @@
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="S130" s="2" t="inlineStr"/>
+      <c r="S130" s="2" t="n">
+        <v>0.1525</v>
+      </c>
       <c r="T130" s="2" t="inlineStr">
         <is>
-          <t>0.1525</t>
+          <t>likely_benign</t>
         </is>
       </c>
       <c r="U130" s="2" t="inlineStr">
@@ -11618,6 +14488,28 @@
         <v>0</v>
       </c>
       <c r="W130" s="2" t="inlineStr"/>
+      <c r="X130" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y130" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z130" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA130" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB130" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC130" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -11686,10 +14578,12 @@
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="S131" s="2" t="inlineStr"/>
+      <c r="S131" s="2" t="n">
+        <v>0.1508</v>
+      </c>
       <c r="T131" s="2" t="inlineStr">
         <is>
-          <t>0.1508</t>
+          <t>likely_benign</t>
         </is>
       </c>
       <c r="U131" s="2" t="inlineStr">
@@ -11701,6 +14595,28 @@
         <v>0</v>
       </c>
       <c r="W131" s="2" t="inlineStr"/>
+      <c r="X131" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y131" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z131" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA131" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB131" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC131" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -11769,10 +14685,12 @@
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="S132" s="2" t="inlineStr"/>
+      <c r="S132" s="2" t="n">
+        <v>0.0679</v>
+      </c>
       <c r="T132" s="2" t="inlineStr">
         <is>
-          <t>0.0679</t>
+          <t>likely_benign</t>
         </is>
       </c>
       <c r="U132" s="2" t="inlineStr">
@@ -11784,6 +14702,28 @@
         <v>0</v>
       </c>
       <c r="W132" s="2" t="inlineStr"/>
+      <c r="X132" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y132" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z132" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA132" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB132" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC132" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -11852,10 +14792,12 @@
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="S133" s="2" t="inlineStr"/>
+      <c r="S133" s="2" t="n">
+        <v>0.2646</v>
+      </c>
       <c r="T133" s="2" t="inlineStr">
         <is>
-          <t>0.2646</t>
+          <t>likely_benign</t>
         </is>
       </c>
       <c r="U133" s="2" t="inlineStr">
@@ -11867,6 +14809,28 @@
         <v>0</v>
       </c>
       <c r="W133" s="2" t="inlineStr"/>
+      <c r="X133" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y133" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z133" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA133" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB133" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC133" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -11935,10 +14899,12 @@
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="S134" s="2" t="inlineStr"/>
+      <c r="S134" s="2" t="n">
+        <v>0.1489</v>
+      </c>
       <c r="T134" s="2" t="inlineStr">
         <is>
-          <t>0.1489</t>
+          <t>likely_benign</t>
         </is>
       </c>
       <c r="U134" s="2" t="inlineStr">
@@ -11950,6 +14916,28 @@
         <v>0</v>
       </c>
       <c r="W134" s="2" t="inlineStr"/>
+      <c r="X134" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y134" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z134" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA134" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB134" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC134" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -12018,10 +15006,12 @@
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="S135" s="2" t="inlineStr"/>
+      <c r="S135" s="2" t="n">
+        <v>0.2344</v>
+      </c>
       <c r="T135" s="2" t="inlineStr">
         <is>
-          <t>0.2344</t>
+          <t>likely_benign</t>
         </is>
       </c>
       <c r="U135" s="2" t="inlineStr">
@@ -12033,6 +15023,28 @@
         <v>0</v>
       </c>
       <c r="W135" s="2" t="inlineStr"/>
+      <c r="X135" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y135" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z135" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA135" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB135" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC135" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -12101,10 +15113,12 @@
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="S136" s="2" t="inlineStr"/>
+      <c r="S136" s="2" t="n">
+        <v>0.0949</v>
+      </c>
       <c r="T136" s="2" t="inlineStr">
         <is>
-          <t>0.0949</t>
+          <t>likely_benign</t>
         </is>
       </c>
       <c r="U136" s="2" t="inlineStr">
@@ -12116,6 +15130,28 @@
         <v>0</v>
       </c>
       <c r="W136" s="2" t="inlineStr"/>
+      <c r="X136" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y136" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z136" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA136" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB136" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC136" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -12201,6 +15237,28 @@
         <v>0</v>
       </c>
       <c r="W137" s="2" t="inlineStr"/>
+      <c r="X137" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y137" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z137" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA137" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB137" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC137" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -12286,6 +15344,28 @@
         <v>0</v>
       </c>
       <c r="W138" s="2" t="inlineStr"/>
+      <c r="X138" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y138" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z138" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA138" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB138" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC138" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -12371,6 +15451,28 @@
         <v>0</v>
       </c>
       <c r="W139" s="2" t="inlineStr"/>
+      <c r="X139" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y139" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z139" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA139" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB139" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC139" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -12456,6 +15558,28 @@
         <v>0</v>
       </c>
       <c r="W140" s="2" t="inlineStr"/>
+      <c r="X140" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y140" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z140" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA140" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB140" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC140" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -12541,6 +15665,28 @@
         <v>0</v>
       </c>
       <c r="W141" s="2" t="inlineStr"/>
+      <c r="X141" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y141" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z141" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA141" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB141" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC141" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -12626,6 +15772,28 @@
         <v>0</v>
       </c>
       <c r="W142" s="2" t="inlineStr"/>
+      <c r="X142" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y142" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z142" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA142" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB142" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC142" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -12711,6 +15879,28 @@
         <v>0</v>
       </c>
       <c r="W143" s="2" t="inlineStr"/>
+      <c r="X143" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y143" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z143" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AA143" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB143" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC143" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -12796,6 +15986,28 @@
         <v>0</v>
       </c>
       <c r="W144" s="2" t="inlineStr"/>
+      <c r="X144" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y144" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z144" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA144" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB144" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC144" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -12881,6 +16093,28 @@
         <v>0</v>
       </c>
       <c r="W145" s="2" t="inlineStr"/>
+      <c r="X145" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y145" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z145" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="AA145" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB145" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC145" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>